<commit_message>
orders-no-desig-assign: updated excel sheet
</commit_message>
<xml_diff>
--- a/order-no-desig-assign/WarehouseDetail_records(order-no-desig-assign).xlsx
+++ b/order-no-desig-assign/WarehouseDetail_records(order-no-desig-assign).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rndc/Desktop/Work related/Documents/order-no-desig-assign/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEDEFD55-87E0-FB47-A740-A5CA0D752D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EB87201-3973-934F-90EC-B56FD7837908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20500" xr2:uid="{00000000-000D-0000-FFFF-FFFF01000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20480" xr2:uid="{00000000-000D-0000-FFFF-FFFF01000000}"/>
   </bookViews>
   <sheets>
     <sheet name="(main group)" sheetId="6" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="178">
   <si>
     <t>Current</t>
   </si>
@@ -1594,7 +1594,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1621,10 +1621,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1962,7 +1958,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A63BE434-9ED0-E94E-BE21-7A21279D6729}">
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="10.1640625" customWidth="1"/>
@@ -1970,7 +1966,7 @@
     <col min="8" max="8" width="17.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>56</v>
       </c>
@@ -2005,7 +2001,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" t="b">
         <v>0</v>
       </c>
@@ -2024,7 +2020,9 @@
       <c r="F2" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G2" s="13"/>
+      <c r="G2" t="s">
+        <v>122</v>
+      </c>
       <c r="H2" s="3" t="s">
         <v>172</v>
       </c>
@@ -2037,9 +2035,9 @@
       <c r="K2" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="L2" s="12"/>
-    </row>
-    <row r="3" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="M2" s="3"/>
+    </row>
+    <row r="3" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" t="b">
         <v>0</v>
       </c>
@@ -2058,7 +2056,9 @@
       <c r="F3" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G3" s="13"/>
+      <c r="G3" t="s">
+        <v>147</v>
+      </c>
       <c r="H3" s="3" t="s">
         <v>172</v>
       </c>
@@ -2071,8 +2071,9 @@
       <c r="K3" s="3" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="M3" s="3"/>
+    </row>
+    <row r="4" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" t="b">
         <v>0</v>
       </c>
@@ -2091,7 +2092,9 @@
       <c r="F4" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G4" s="13"/>
+      <c r="G4" t="s">
+        <v>123</v>
+      </c>
       <c r="H4" s="3" t="s">
         <v>172</v>
       </c>
@@ -2104,9 +2107,9 @@
       <c r="K4" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="L4" s="3"/>
-    </row>
-    <row r="5" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="M4" s="3"/>
+    </row>
+    <row r="5" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" t="b">
         <v>0</v>
       </c>
@@ -2125,7 +2128,9 @@
       <c r="F5" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G5" s="13"/>
+      <c r="G5" t="s">
+        <v>124</v>
+      </c>
       <c r="H5" s="3" t="s">
         <v>172</v>
       </c>
@@ -2138,8 +2143,9 @@
       <c r="K5" s="3" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="M5" s="3"/>
+    </row>
+    <row r="6" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" t="b">
         <v>0</v>
       </c>
@@ -2158,7 +2164,9 @@
       <c r="F6" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G6" s="13"/>
+      <c r="G6" t="s">
+        <v>148</v>
+      </c>
       <c r="H6" s="3" t="s">
         <v>172</v>
       </c>
@@ -2172,7 +2180,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" t="b">
         <v>0</v>
       </c>
@@ -2191,7 +2199,9 @@
       <c r="F7" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G7" s="13"/>
+      <c r="G7" t="s">
+        <v>159</v>
+      </c>
       <c r="H7" s="3" t="s">
         <v>172</v>
       </c>
@@ -2205,7 +2215,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" t="b">
         <v>0</v>
       </c>
@@ -2224,7 +2234,9 @@
       <c r="F8" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G8" s="13"/>
+      <c r="G8" t="s">
+        <v>160</v>
+      </c>
       <c r="H8" s="3" t="s">
         <v>172</v>
       </c>
@@ -2238,7 +2250,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A9" t="b">
         <v>0</v>
       </c>
@@ -2257,7 +2269,9 @@
       <c r="F9" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G9" s="13"/>
+      <c r="G9" t="s">
+        <v>161</v>
+      </c>
       <c r="H9" s="3" t="s">
         <v>172</v>
       </c>
@@ -2270,8 +2284,9 @@
       <c r="K9" s="3" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="M9" s="3"/>
+    </row>
+    <row r="10" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" t="b">
         <v>0</v>
       </c>
@@ -2290,7 +2305,9 @@
       <c r="F10" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G10" s="13"/>
+      <c r="G10" t="s">
+        <v>125</v>
+      </c>
       <c r="H10" s="3" t="s">
         <v>172</v>
       </c>
@@ -2303,8 +2320,9 @@
       <c r="K10" s="3" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="M10" s="3"/>
+    </row>
+    <row r="11" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A11" t="b">
         <v>0</v>
       </c>
@@ -2323,7 +2341,9 @@
       <c r="F11" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G11" s="13"/>
+      <c r="G11" t="s">
+        <v>126</v>
+      </c>
       <c r="H11" s="3" t="s">
         <v>172</v>
       </c>
@@ -2337,7 +2357,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" t="b">
         <v>0</v>
       </c>
@@ -2356,7 +2376,9 @@
       <c r="F12" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G12" s="13"/>
+      <c r="G12" t="s">
+        <v>127</v>
+      </c>
       <c r="H12" s="3" t="s">
         <v>172</v>
       </c>
@@ -2370,7 +2392,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" t="b">
         <v>0</v>
       </c>
@@ -2389,7 +2411,9 @@
       <c r="F13" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G13" s="13"/>
+      <c r="G13" t="s">
+        <v>128</v>
+      </c>
       <c r="H13" s="3" t="s">
         <v>172</v>
       </c>
@@ -2403,7 +2427,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" t="b">
         <v>0</v>
       </c>
@@ -2422,7 +2446,9 @@
       <c r="F14" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G14" s="13"/>
+      <c r="G14" t="s">
+        <v>129</v>
+      </c>
       <c r="H14" s="3" t="s">
         <v>172</v>
       </c>
@@ -2436,7 +2462,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" t="b">
         <v>0</v>
       </c>
@@ -2455,7 +2481,9 @@
       <c r="F15" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G15" s="13"/>
+      <c r="G15" t="s">
+        <v>130</v>
+      </c>
       <c r="H15" s="3" t="s">
         <v>172</v>
       </c>
@@ -2469,7 +2497,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" t="b">
         <v>0</v>
       </c>
@@ -2488,7 +2516,9 @@
       <c r="F16" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G16" s="13"/>
+      <c r="G16" t="s">
+        <v>156</v>
+      </c>
       <c r="H16" s="3" t="s">
         <v>172</v>
       </c>
@@ -2502,7 +2532,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A17" t="b">
         <v>0</v>
       </c>
@@ -2521,7 +2551,9 @@
       <c r="F17" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G17" s="13"/>
+      <c r="G17" t="s">
+        <v>131</v>
+      </c>
       <c r="H17" s="3" t="s">
         <v>172</v>
       </c>
@@ -2535,7 +2567,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" t="b">
         <v>0</v>
       </c>
@@ -2554,7 +2586,9 @@
       <c r="F18" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G18" s="13"/>
+      <c r="G18" t="s">
+        <v>132</v>
+      </c>
       <c r="H18" s="3" t="s">
         <v>172</v>
       </c>
@@ -2568,7 +2602,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" t="b">
         <v>0</v>
       </c>
@@ -2587,7 +2621,9 @@
       <c r="F19" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G19" s="13"/>
+      <c r="G19" t="s">
+        <v>133</v>
+      </c>
       <c r="H19" s="3" t="s">
         <v>172</v>
       </c>
@@ -2601,7 +2637,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" t="b">
         <v>0</v>
       </c>
@@ -2620,7 +2656,9 @@
       <c r="F20" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G20" s="13"/>
+      <c r="G20" t="s">
+        <v>134</v>
+      </c>
       <c r="H20" s="3" t="s">
         <v>172</v>
       </c>
@@ -2634,7 +2672,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" t="b">
         <v>0</v>
       </c>
@@ -2653,7 +2691,9 @@
       <c r="F21" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G21" s="13"/>
+      <c r="G21" t="s">
+        <v>153</v>
+      </c>
       <c r="H21" s="3" t="s">
         <v>172</v>
       </c>
@@ -2667,7 +2707,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" t="b">
         <v>0</v>
       </c>
@@ -2686,7 +2726,9 @@
       <c r="F22" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G22" s="13"/>
+      <c r="G22" t="s">
+        <v>155</v>
+      </c>
       <c r="H22" s="3" t="s">
         <v>172</v>
       </c>
@@ -2700,7 +2742,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" t="b">
         <v>0</v>
       </c>
@@ -2719,7 +2761,9 @@
       <c r="F23" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G23" s="13"/>
+      <c r="G23" t="s">
+        <v>135</v>
+      </c>
       <c r="H23" s="3" t="s">
         <v>172</v>
       </c>
@@ -2733,7 +2777,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A24" t="b">
         <v>0</v>
       </c>
@@ -2752,7 +2796,9 @@
       <c r="F24" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G24" s="13"/>
+      <c r="G24" t="s">
+        <v>136</v>
+      </c>
       <c r="H24" s="3" t="s">
         <v>172</v>
       </c>
@@ -2766,7 +2812,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A25" t="b">
         <v>0</v>
       </c>
@@ -2785,7 +2831,9 @@
       <c r="F25" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G25" s="13"/>
+      <c r="G25" t="s">
+        <v>149</v>
+      </c>
       <c r="H25" s="3" t="s">
         <v>172</v>
       </c>
@@ -2798,8 +2846,9 @@
       <c r="K25" s="3" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+      <c r="M25" s="3"/>
+    </row>
+    <row r="26" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A26" t="b">
         <v>0</v>
       </c>
@@ -2818,7 +2867,9 @@
       <c r="F26" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G26" s="13"/>
+      <c r="G26" t="s">
+        <v>150</v>
+      </c>
       <c r="H26" s="3" t="s">
         <v>172</v>
       </c>
@@ -2832,7 +2883,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A27" t="b">
         <v>0</v>
       </c>
@@ -2851,7 +2902,9 @@
       <c r="F27" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G27" s="13"/>
+      <c r="G27" t="s">
+        <v>154</v>
+      </c>
       <c r="H27" s="3" t="s">
         <v>172</v>
       </c>
@@ -2865,7 +2918,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A28" t="b">
         <v>0</v>
       </c>
@@ -2884,7 +2937,9 @@
       <c r="F28" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G28" s="13"/>
+      <c r="G28" t="s">
+        <v>137</v>
+      </c>
       <c r="H28" s="3" t="s">
         <v>172</v>
       </c>
@@ -2898,7 +2953,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A29" t="b">
         <v>0</v>
       </c>
@@ -2917,7 +2972,9 @@
       <c r="F29" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G29" s="13"/>
+      <c r="G29" t="s">
+        <v>152</v>
+      </c>
       <c r="H29" s="3" t="s">
         <v>172</v>
       </c>
@@ -2931,7 +2988,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A30" t="b">
         <v>0</v>
       </c>
@@ -2950,7 +3007,9 @@
       <c r="F30" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G30" s="13"/>
+      <c r="G30" t="s">
+        <v>138</v>
+      </c>
       <c r="H30" s="3" t="s">
         <v>172</v>
       </c>
@@ -2964,7 +3023,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A31" t="b">
         <v>0</v>
       </c>
@@ -2983,7 +3042,9 @@
       <c r="F31" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G31" s="13"/>
+      <c r="G31" t="s">
+        <v>139</v>
+      </c>
       <c r="H31" s="3" t="s">
         <v>172</v>
       </c>
@@ -2997,7 +3058,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" t="b">
         <v>0</v>
       </c>
@@ -3016,7 +3077,9 @@
       <c r="F32" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G32" s="13"/>
+      <c r="G32" t="s">
+        <v>140</v>
+      </c>
       <c r="H32" s="3" t="s">
         <v>172</v>
       </c>
@@ -3030,7 +3093,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A33" t="b">
         <v>0</v>
       </c>
@@ -3049,7 +3112,9 @@
       <c r="F33" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G33" s="13"/>
+      <c r="G33" t="s">
+        <v>141</v>
+      </c>
       <c r="H33" s="3" t="s">
         <v>172</v>
       </c>
@@ -3062,8 +3127,9 @@
       <c r="K33" s="3" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="34" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+      <c r="M33" s="3"/>
+    </row>
+    <row r="34" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A34" t="b">
         <v>0</v>
       </c>
@@ -3082,7 +3148,9 @@
       <c r="F34" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G34" s="13"/>
+      <c r="G34" t="s">
+        <v>162</v>
+      </c>
       <c r="H34" s="3" t="s">
         <v>172</v>
       </c>
@@ -3096,7 +3164,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" t="b">
         <v>0</v>
       </c>
@@ -3115,7 +3183,9 @@
       <c r="F35" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G35" s="13"/>
+      <c r="G35" t="s">
+        <v>142</v>
+      </c>
       <c r="H35" s="3" t="s">
         <v>172</v>
       </c>
@@ -3128,8 +3198,9 @@
       <c r="K35" s="3" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="36" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+      <c r="M35" s="3"/>
+    </row>
+    <row r="36" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A36" t="b">
         <v>1</v>
       </c>
@@ -3148,7 +3219,9 @@
       <c r="F36" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G36" s="12"/>
+      <c r="G36" t="s">
+        <v>121</v>
+      </c>
       <c r="H36" s="3" t="s">
         <v>172</v>
       </c>
@@ -3162,7 +3235,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A37" t="b">
         <v>0</v>
       </c>
@@ -3181,7 +3254,9 @@
       <c r="F37" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G37" s="13"/>
+      <c r="G37" t="s">
+        <v>157</v>
+      </c>
       <c r="H37" s="3" t="s">
         <v>172</v>
       </c>
@@ -3195,7 +3270,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" t="b">
         <v>0</v>
       </c>
@@ -3214,7 +3289,9 @@
       <c r="F38" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G38" s="13"/>
+      <c r="G38" t="s">
+        <v>151</v>
+      </c>
       <c r="H38" s="3" t="s">
         <v>172</v>
       </c>
@@ -3227,8 +3304,9 @@
       <c r="K38" s="3" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="39" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+      <c r="M38" s="3"/>
+    </row>
+    <row r="39" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" t="b">
         <v>0</v>
       </c>
@@ -3247,7 +3325,9 @@
       <c r="F39" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G39" s="13"/>
+      <c r="G39" t="s">
+        <v>143</v>
+      </c>
       <c r="H39" s="3" t="s">
         <v>172</v>
       </c>
@@ -3261,7 +3341,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" t="b">
         <v>0</v>
       </c>
@@ -3280,7 +3360,9 @@
       <c r="F40" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G40" s="13"/>
+      <c r="G40" t="s">
+        <v>144</v>
+      </c>
       <c r="H40" s="3" t="s">
         <v>172</v>
       </c>
@@ -3294,7 +3376,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A41" t="b">
         <v>0</v>
       </c>
@@ -3313,7 +3395,9 @@
       <c r="F41" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G41" s="13"/>
+      <c r="G41" t="s">
+        <v>145</v>
+      </c>
       <c r="H41" s="3" t="s">
         <v>172</v>
       </c>
@@ -3327,7 +3411,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" t="b">
         <v>0</v>
       </c>
@@ -3346,7 +3430,9 @@
       <c r="F42" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G42" s="13"/>
+      <c r="G42" t="s">
+        <v>163</v>
+      </c>
       <c r="H42" s="3" t="s">
         <v>172</v>
       </c>
@@ -3360,7 +3446,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" t="b">
         <v>0</v>
       </c>
@@ -3379,7 +3465,9 @@
       <c r="F43" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G43" s="13"/>
+      <c r="G43" t="s">
+        <v>158</v>
+      </c>
       <c r="H43" s="3" t="s">
         <v>172</v>
       </c>
@@ -3393,7 +3481,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" t="b">
         <v>0</v>
       </c>
@@ -3412,7 +3500,9 @@
       <c r="F44" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G44" s="13"/>
+      <c r="G44" t="s">
+        <v>146</v>
+      </c>
       <c r="H44" s="3" t="s">
         <v>172</v>
       </c>
@@ -3433,7 +3523,7 @@
       <c r="D51" s="11"/>
     </row>
     <row r="52" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C52" s="14">
+      <c r="C52" s="12">
         <v>1</v>
       </c>
       <c r="D52" s="11" t="s">
@@ -3441,7 +3531,7 @@
       </c>
     </row>
     <row r="53" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C53" s="14">
+      <c r="C53" s="12">
         <v>40</v>
       </c>
       <c r="D53" s="11" t="s">

</xml_diff>